<commit_message>
Fix footwork trigger status
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -53345,7 +53345,7 @@
       </c>
       <c r="O807" s="18" t="inlineStr">
         <is>
-          <t>Secondary effect not possible with mechanical system // Developer follow-up (2026-07-19): The secondary effect is implemented as +6% Evasion for 30 seconds and is covered by static validation. Live retest required.</t>
+          <t>Secondary effect not possible with mechanical system // Developer follow-up (2026-07-19): The secondary effect is implemented as +6% Evasion for 30 seconds and is covered by static validation. Live retest required. // External report review (2026-07-19): This report predates the comprehensive review. Verified that rank I has one normal 3 STM cost and automatically grants +6% Evasion for 30 seconds; there is no additional-cost toggle. Static regression passed; live retest remains required.</t>
         </is>
       </c>
     </row>
@@ -53420,7 +53420,7 @@
       </c>
       <c r="O808" s="18" t="inlineStr">
         <is>
-          <t>Did not grant evasion on trigger // Developer follow-up (2026-07-19): Fixed missing stat wiring. It now grants +10% Evasion for 30 seconds after any Spear ability, matching the current Bible description.</t>
+          <t>Did not grant evasion on trigger // Developer follow-up (2026-07-19): Fixed missing stat wiring. It now grants +10% Evasion for 30 seconds after any Spear ability, matching the current Bible description. // External report review (2026-07-19): The missing Evasion wiring had already been fixed. Added a visible Evasive Footwork status that grants +10% Evasion for 30 seconds, refreshes after any Spear ability, and uses a unique beneficial status icon. Static regression passed; live retest remains required. // Cross-skill follow-up (2026-07-19): Isolated Pistol Mobile Footwork and Spear Lateral Footwork selector channels so owning both cannot sum skill IDs and disable both. Their shared status refreshes instead of stacking.</t>
         </is>
       </c>
     </row>
@@ -53645,7 +53645,7 @@
       </c>
       <c r="O811" s="18" t="inlineStr">
         <is>
-          <t>Secondary effect not possible with mechanical system // Developer follow-up (2026-07-19): The secondary effect is implemented as +8% Evasion for 30 seconds and is covered by static validation. Live retest required.</t>
+          <t>Secondary effect not possible with mechanical system // Developer follow-up (2026-07-19): The secondary effect is implemented as +8% Evasion for 30 seconds and is covered by static validation. Live retest required. // External report review (2026-07-19): This report predates the comprehensive review. Verified that rank II has one normal 5 STM cost and automatically grants +8% Evasion for 30 seconds; there is no additional-cost toggle. Static regression passed; live retest remains required.</t>
         </is>
       </c>
     </row>
@@ -54089,7 +54089,7 @@
       </c>
       <c r="O817" s="18" t="inlineStr">
         <is>
-          <t>Secondary effect not possible with mechanical system // Developer follow-up (2026-07-19): The secondary effect is implemented as +10% Evasion for 30 seconds and is covered by static validation. Live retest required.</t>
+          <t>Secondary effect not possible with mechanical system // Developer follow-up (2026-07-19): The secondary effect is implemented as +10% Evasion for 30 seconds and is covered by static validation. Live retest required. // External report review (2026-07-19): This report predates the comprehensive review. Verified that rank III has one normal 8 STM cost and automatically grants +10% Evasion for 30 seconds; there is no additional-cost toggle. Static regression passed; live retest remains required.</t>
         </is>
       </c>
     </row>
@@ -54461,7 +54461,7 @@
       </c>
       <c r="O822" s="18" t="inlineStr">
         <is>
-          <t>Secondary effect not possible with mechanical system // Developer follow-up (2026-07-19): The secondary effect is implemented as +12% Evasion for 30 seconds and is covered by static validation. Live retest required.</t>
+          <t>Secondary effect not possible with mechanical system // Developer follow-up (2026-07-19): The secondary effect is implemented as +12% Evasion for 30 seconds and is covered by static validation. Live retest required. // External report review (2026-07-19): This report predates the comprehensive review. Verified that rank IV has one normal 12 STM cost and automatically grants +12% Evasion for 30 seconds; there is no additional-cost toggle. Static regression passed; live retest remains required.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix global Vigor Stance effects
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -53823,7 +53823,7 @@
       </c>
       <c r="F814" s="4" t="inlineStr">
         <is>
-          <t>While active, hostile combat abilities cost 2 additional STM, deal +10% damage, and grant +8% Evasion for 30 seconds.</t>
+          <t>While active, all outgoing damage is increased by 10%. Using any hostile combat ability costs 2 additional STM and grants +8% Evasion for 30 seconds.</t>
         </is>
       </c>
       <c r="G814" s="3" t="inlineStr">
@@ -53866,7 +53866,7 @@
       </c>
       <c r="O814" s="18" t="inlineStr">
         <is>
-          <t>No Stamina cost increase, no Damage increase, no Evasion increase // Developer follow-up (2026-07-19): Fixed all three payloads: +2 STM cost, +10% Spear ability damage inside the shared damage cap, and +8% Evasion for 30 seconds after hostile Spear abilities. Independent trigger channels prevent invalid stacking.</t>
+          <t>No Stamina cost increase, no Damage increase, no Evasion increase // Developer follow-up (2026-07-19): Vigor Stance is now global as intended: +10% all outgoing damage, +2 STM on every hostile combat ability, and +8% Evasion for 30 seconds after any hostile combat ability. The Character Sheet now refreshes when temporary stat modifiers start or expire, and the outgoing-damage cap plus independent refresh channel prevent unbounded stacking.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix High Guard costly ability interactions
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -53495,7 +53495,7 @@
       </c>
       <c r="O809" s="18" t="inlineStr">
         <is>
-          <t>Did not grant evasion on trigger // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +3% Evasion for 30 seconds; damage remains +6.</t>
+          <t>Did not grant evasion on trigger // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +3% Evasion for 30 seconds; damage remains +6. // Developer correction (2026-07-19): The earlier fix was incomplete. Restoration Strike consumed the paid-cost context before High Guard Evasion ran, while shared minimum-cost stats made High Guard damage, Restoration Strike, and Crippling Defense thresholds add together. The cost is now bound to the exact ability, remains available to every independent rider, restores STM only once, and uses separate 8 STM thresholds. High Guard now applies globally per the Bible wording. Retest with Restoration Strike and Crippling Defense owned, using any hostile ability that spends at least 8 final STM.</t>
         </is>
       </c>
     </row>
@@ -53941,7 +53941,7 @@
       </c>
       <c r="O815" s="18" t="inlineStr">
         <is>
-          <t>No evasion increase, no way to tell DMG increased // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +5% Evasion for 30 seconds; damage remains +10.</t>
+          <t>No evasion increase, no way to tell DMG increased // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +5% Evasion for 30 seconds; damage remains +10. // Developer correction (2026-07-19): The earlier fix was incomplete. Restoration Strike consumed the paid-cost context before High Guard Evasion ran, while shared minimum-cost stats made High Guard damage, Restoration Strike, and Crippling Defense thresholds add together. The cost is now bound to the exact ability, remains available to every independent rider, restores STM only once, and uses separate 8 STM thresholds. High Guard now applies globally per the Bible wording. Retest with Restoration Strike and Crippling Defense owned, using any hostile ability that spends at least 8 final STM.</t>
         </is>
       </c>
     </row>
@@ -54003,7 +54003,7 @@
       </c>
       <c r="L816" s="12" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M816" s="13" t="inlineStr">
@@ -54015,7 +54015,11 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Fill with today's date"")"),"2026-07-18")</f>
         <v/>
       </c>
-      <c r="O816" s="18" t="n"/>
+      <c r="O816" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Corrected an interaction bug in the shared costly-ability context. Restoration Strike no longer raises High Guard's damage threshold, no longer consumes High Guard's Evasion trigger, restores 3 STM only once per ability, and now applies to any hostile ability spending at least 8 final STM as written. Retest together with High Guard and a multi-target ability.</t>
+        </is>
+      </c>
     </row>
     <row r="817" ht="15" customHeight="1" s="16">
       <c r="A817" s="9" t="inlineStr">
@@ -54537,7 +54541,7 @@
       </c>
       <c r="O823" s="18" t="inlineStr">
         <is>
-          <t>No evasion increase, no way to tell DMG increased // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +7% Evasion for 30 seconds; damage remains +14.</t>
+          <t>No evasion increase, no way to tell DMG increased // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +7% Evasion for 30 seconds; damage remains +14. // Developer correction (2026-07-19): The earlier fix was incomplete. Restoration Strike consumed the paid-cost context before High Guard Evasion ran, while shared minimum-cost stats made High Guard damage, Restoration Strike, and Crippling Defense thresholds add together. The cost is now bound to the exact ability, remains available to every independent rider, restores STM only once, and uses separate 8 STM thresholds. High Guard now applies globally per the Bible wording. Retest with Restoration Strike and Crippling Defense owned, using any hostile ability that spends at least 8 final STM.</t>
         </is>
       </c>
     </row>
@@ -54613,7 +54617,7 @@
       </c>
       <c r="O824" s="18" t="inlineStr">
         <is>
-          <t>Ability locked // Developer follow-up (2026-07-19): No defect identified; this is the intended capstone quest gate. Retest with the quest completed or an approved admin test fixture.</t>
+          <t>Ability locked // Developer follow-up (2026-07-19): No defect identified; this is the intended capstone quest gate. Retest with the quest completed or an approved admin test fixture. // Developer follow-up (2026-07-19): Its 8 STM Exposed threshold is now independent rather than adding to High Guard/Restoration thresholds, and “high-STM abilities” is global per the Bible. Keep Blocked until capstone access is available; then retest alongside High Guard and Restoration Strike.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix stealth and outstanding combat test feedback
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -1280,7 +1280,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Increases Detection by 5, improving your chance to notice stealthed creatures.</t>
+          <t>Increases Detection by 10, improving your chance to notice stealthed creatures.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1310,12 +1310,16 @@
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M12" s="13" t="n"/>
       <c r="N12" s="14" t="n"/>
-      <c r="O12" s="18" t="n"/>
+      <c r="O12" s="18" t="inlineStr">
+        <is>
+          <t>Retest Detection = PER + WIL + equipment/status bonuses + 10 Alertness; Detect mode adds +5. Validate against all Stealth ranks at close and long visual range.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="16">
       <c r="A13" s="9" t="inlineStr">
@@ -1345,7 +1349,7 @@
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>Increases Detection by 10, improving your chance to notice stealthed creatures.</t>
+          <t>Increases Detection by 15, improving your chance to notice stealthed creatures.</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -1375,12 +1379,16 @@
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M13" s="13" t="n"/>
       <c r="N13" s="14" t="n"/>
-      <c r="O13" s="18" t="n"/>
+      <c r="O13" s="18" t="inlineStr">
+        <is>
+          <t>Retest Detection = PER + WIL + equipment/status bonuses + 15 Alertness; Detect mode adds +5. Validate against all Stealth ranks at close and long visual range.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="16">
       <c r="A14" s="2" t="inlineStr">
@@ -1410,7 +1418,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Increases Detection by 15, improving your chance to notice stealthed creatures.</t>
+          <t>Increases Detection by 20, improving your chance to notice stealthed creatures.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1440,12 +1448,16 @@
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="14" t="n"/>
-      <c r="O14" s="18" t="n"/>
+      <c r="O14" s="18" t="inlineStr">
+        <is>
+          <t>Retest Detection = PER + WIL + equipment/status bonuses + 20 Alertness; Detect mode adds +5. Validate that a fully committed spotter can counter a fully committed stealther.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="16">
       <c r="A15" s="9" t="inlineStr">
@@ -13284,7 +13296,11 @@
       <c r="N196" s="14" t="n">
         <v>46221</v>
       </c>
-      <c r="O196" s="18" t="n"/>
+      <c r="O196" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed intentional: Flamethrower I deals cone fire damage but does not apply Burn. Burn begins at Flamethrower II per the current Bible.</t>
+        </is>
+      </c>
     </row>
     <row r="197" ht="15" customHeight="1" s="16">
       <c r="A197" s="9" t="inlineStr">
@@ -13503,7 +13519,7 @@
       </c>
       <c r="O199" s="18" t="inlineStr">
         <is>
-          <t>Accuracy increase works, unclear if the crit boost does // Developer follow-up (2026-07-19): Verified +8% Assault Gadget Accuracy and +8% critical chance are consumed by every damaging Assault Gadget definition. Retest critical frequency with and without the perk.</t>
+          <t>Developer follow-up (2026-07-19): Fixed ability critical math so the 5% baseline and +8% Gadget Harness stack to 13% total. The Character Sheet now shows Assault Gadget Crit, and successful ability criticals print an identity-safe 'critically hits' combat message. With Tactical Uplink active, the displayed total should be 18%. Retest the readout and critical frequency over a large sample.</t>
         </is>
       </c>
     </row>
@@ -13649,7 +13665,7 @@
       </c>
       <c r="O201" s="18" t="inlineStr">
         <is>
-          <t>Burn effect seems to only last 1 round, burn duration not listed in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Burn (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Burn at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Flamethrower II on successful Burn applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -13795,7 +13811,7 @@
       </c>
       <c r="O203" s="18" t="inlineStr">
         <is>
-          <t>Bleed effect applies for 1 round, bleed duration not stated in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Bleed (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Bleed at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Rail Dart I on successful Bleed applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -13870,7 +13886,7 @@
       </c>
       <c r="O204" s="18" t="inlineStr">
         <is>
-          <t>Accuracy increase works, unclear if the crit boost does // Developer follow-up (2026-07-19): Verified the 30-second buff supplies +5% Devices ability Accuracy and +5% Devices ability critical chance, and Assault Gadgets consume both. Retest critical frequency with and without the buff.</t>
+          <t>Developer follow-up (2026-07-19): Fixed ability critical math so Tactical Uplink adds +5 points to the 5% baseline (10% without Gadget Harness; 18% with Harness). The Character Sheet Assault Gadget Crit row updates with the buff, and successful ability criticals print an identity-safe combat message. Retest the 30-second buff, readout, and critical frequency.</t>
         </is>
       </c>
     </row>
@@ -14304,7 +14320,7 @@
       </c>
       <c r="O210" s="18" t="inlineStr">
         <is>
-          <t>Burn effect seems to only last 1 round, burn duration not listed in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Burn (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Burn at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Flamethrower III on successful Burn applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -14379,7 +14395,7 @@
       </c>
       <c r="O211" s="18" t="inlineStr">
         <is>
-          <t>Bleed effect applies for 1 round, bleed duration not stated in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Bleed (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Bleed at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Rail Dart II on successful Bleed applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -14600,7 +14616,7 @@
       </c>
       <c r="O214" s="18" t="inlineStr">
         <is>
-          <t>Bleed effect applies for 1 round, bleed duration not stated in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Bleed (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Bleed at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Rail Dart III on successful Bleed applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15516,7 @@
       </c>
       <c r="F228" s="4" t="inlineStr">
         <is>
-          <t>Enter stealth, increasing stealth effectiveness by 15% while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
+          <t>Enter stealth, increasing Stealth by 5 while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
         </is>
       </c>
       <c r="G228" s="3" t="inlineStr">
@@ -15530,12 +15546,16 @@
       </c>
       <c r="L228" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M228" s="13" t="n"/>
       <c r="N228" s="14" t="n"/>
-      <c r="O228" s="18" t="n"/>
+      <c r="O228" s="18" t="inlineStr">
+        <is>
+          <t>Retest base Stealth without the perk (no mode, status, or STM drain), perk toggle on/off, clean in-combat rejection, icon/drain cleanup, and Stealth = (AGI x 2) + equipment/status + 5.</t>
+        </is>
+      </c>
     </row>
     <row r="229" ht="15" customHeight="1" s="16">
       <c r="A229" s="9" t="inlineStr">
@@ -15760,7 +15780,7 @@
       </c>
       <c r="F232" s="4" t="inlineStr">
         <is>
-          <t>Enter stealth, increasing stealth effectiveness by 25% while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
+          <t>Enter stealth, increasing Stealth by 10 while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
         </is>
       </c>
       <c r="G232" s="3" t="inlineStr">
@@ -15790,12 +15810,16 @@
       </c>
       <c r="L232" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M232" s="13" t="n"/>
       <c r="N232" s="14" t="n"/>
-      <c r="O232" s="18" t="n"/>
+      <c r="O232" s="18" t="inlineStr">
+        <is>
+          <t>Retest toggle, clean in-combat rejection, icon/drain cleanup, hostile-action break, and Stealth = (AGI x 2) + equipment/status + 10.</t>
+        </is>
+      </c>
     </row>
     <row r="233" ht="15" customHeight="1" s="16">
       <c r="A233" s="9" t="inlineStr">
@@ -16020,7 +16044,7 @@
       </c>
       <c r="F236" s="4" t="inlineStr">
         <is>
-          <t>Enter stealth, increasing stealth effectiveness by 35% while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
+          <t>Enter stealth, increasing Stealth by 15 while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
         </is>
       </c>
       <c r="G236" s="3" t="inlineStr">
@@ -16050,12 +16074,16 @@
       </c>
       <c r="L236" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M236" s="13" t="n"/>
       <c r="N236" s="14" t="n"/>
-      <c r="O236" s="18" t="n"/>
+      <c r="O236" s="18" t="inlineStr">
+        <is>
+          <t>Retest toggle, clean in-combat rejection, icon/drain cleanup, hostile-action break, and Stealth = (AGI x 2) + equipment/status + 15 against groups of observers.</t>
+        </is>
+      </c>
     </row>
     <row r="237" ht="15" customHeight="1" s="16">
       <c r="A237" s="9" t="inlineStr">
@@ -16150,7 +16178,7 @@
       </c>
       <c r="F238" s="4" t="inlineStr">
         <is>
-          <t>Removes the movement-speed penalty from stealth and reduces its STM drain rate by 20%, from 2 STM every 6 seconds to 2 STM every 7.5 seconds.</t>
+          <t>While stealthed, increases Movement Speed by 30% and reduces STM drain by 20%, from 2 STM every 6 seconds to 2 STM every 7.5 seconds. Stealth still prevents running at full speed.</t>
         </is>
       </c>
       <c r="G238" s="3" t="inlineStr">
@@ -16180,12 +16208,16 @@
       </c>
       <c r="L238" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M238" s="13" t="n"/>
       <c r="N238" s="14" t="n"/>
-      <c r="O238" s="18" t="n"/>
+      <c r="O238" s="18" t="inlineStr">
+        <is>
+          <t>Retest immediate +30% Movement Speed on entering stealth without toggling walk, removal on stealth exit, retained running restriction, and 2 STM drain every 7.5 seconds.</t>
+        </is>
+      </c>
     </row>
     <row r="239" ht="15" customHeight="1" s="16">
       <c r="A239" s="9" t="inlineStr">
@@ -16345,7 +16377,7 @@
       </c>
       <c r="F241" s="17" t="inlineStr">
         <is>
-          <t>Enter stealth, increasing stealth effectiveness by 45% while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
+          <t>Enter stealth, increasing Stealth by 20 while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
         </is>
       </c>
       <c r="G241" s="10" t="inlineStr">
@@ -16375,12 +16407,16 @@
       </c>
       <c r="L241" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M241" s="13" t="n"/>
       <c r="N241" s="14" t="n"/>
-      <c r="O241" s="18" t="n"/>
+      <c r="O241" s="18" t="inlineStr">
+        <is>
+          <t>Retest toggle, clean in-combat rejection, icon/drain cleanup, hostile-action break, and Stealth = (AGI x 2) + equipment/status + 20. Validate committed stealth versus baseline monsters and committed spotters.</t>
+        </is>
+      </c>
     </row>
     <row r="242" ht="15" customHeight="1" s="16">
       <c r="A242" s="2" t="inlineStr">
@@ -16635,12 +16671,16 @@
       </c>
       <c r="L245" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M245" s="13" t="n"/>
       <c r="N245" s="14" t="n"/>
-      <c r="O245" s="18" t="n"/>
+      <c r="O245" s="18" t="inlineStr">
+        <is>
+          <t>Retest in-combat stealth entry through the explicit Ghost Protocol window, 30-second exit, status/icon cleanup, and the revised Stealth/Detection ratings.</t>
+        </is>
+      </c>
     </row>
     <row r="246" ht="15" customHeight="1" s="16">
       <c r="A246" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Fix guard counters and aimed area targeting
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -10749,12 +10749,16 @@
       </c>
       <c r="L157" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M157" s="13" t="n"/>
       <c r="N157" s="14" t="n"/>
-      <c r="O157" s="18" t="n"/>
+      <c r="O157" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Fixed the aimed-area activation contract. Adhesive Grenade I now explicitly requires the selected ground target supplied by its cursor; self-centered execution is rejected. Retest ground placement, the 4m blast, and the five-target cap.</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="15" customHeight="1" s="16">
       <c r="A158" s="2" t="inlineStr">
@@ -11140,12 +11144,16 @@
       </c>
       <c r="L163" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M163" s="13" t="n"/>
       <c r="N163" s="14" t="n"/>
-      <c r="O163" s="18" t="n"/>
+      <c r="O163" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Fixed the aimed-area activation contract. Adhesive Grenade II now explicitly requires the selected ground target supplied by its cursor; self-centered execution is rejected. Retest ground placement, the 4m blast, and the five-target cap.</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="15" customHeight="1" s="16">
       <c r="A164" s="2" t="inlineStr">
@@ -29456,7 +29464,7 @@
       </c>
       <c r="F442" s="4" t="inlineStr">
         <is>
-          <t>Your next attack deals weapon DMG + 8. If you guarded an attack within the last 30 seconds, this deals weapon DMG + 16 instead.</t>
+          <t>Queue your next auto attack to deal weapon DMG + 8. If you guarded an attack within the last 30 seconds, it deals weapon DMG + 16 instead.</t>
         </is>
       </c>
       <c r="G442" s="3" t="inlineStr">
@@ -29471,7 +29479,7 @@
       </c>
       <c r="I442" s="3" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Queued</t>
         </is>
       </c>
       <c r="J442" s="3" t="inlineStr">
@@ -29486,7 +29494,7 @@
       </c>
       <c r="L442" s="12" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M442" s="13" t="inlineStr">
@@ -29498,7 +29506,11 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Add today's current date"")"),"2026-07-18")</f>
         <v/>
       </c>
-      <c r="O442" s="18" t="n"/>
+      <c r="O442" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Converted from a click-targeted activation to a self-queued weapon ability. It now applies to the next landed auto attack and no longer displays a target cursor. Regression retest required.</t>
+        </is>
+      </c>
     </row>
     <row r="443" ht="15" customHeight="1" s="16">
       <c r="A443" s="9" t="inlineStr">
@@ -29600,7 +29612,7 @@
       </c>
       <c r="F444" s="4" t="inlineStr">
         <is>
-          <t>When you guard an attack, your next Katar attack within 30 seconds gains +10% critical chance and deals +10 DMG.</t>
+          <t>When you guard an attack, your next attack within 30 seconds gains +10% critical chance and deals +10 DMG.</t>
         </is>
       </c>
       <c r="G444" s="3" t="inlineStr">
@@ -29644,7 +29656,7 @@
       </c>
       <c r="O444" s="18" t="inlineStr">
         <is>
-          <t>No feedback to tell if triggering // Developer follow-up (2026-07-19): Added explicit 'Counter Ready' feedback. Also fixed its selector collision with Retaliatory Flow so both perks combine as +18 DMG and +10% critical chance instead of producing an invalid skill ID.</t>
+          <t>No feedback to tell if triggering // Developer follow-up (2026-07-19): Added explicit 'Counter Ready' feedback. Also fixed its selector collision with Retaliatory Flow so both perks combine as +18 DMG and +10% critical chance instead of producing an invalid skill ID. // Developer follow-up (2026-07-19): Reworked the trigger to be cross-skill. Guard now arms the next hostile combat ability from any skill with +10 DMG and +10% critical chance for 30 seconds; friendly/self abilities do not consume it. Regression retest required.</t>
         </is>
       </c>
     </row>
@@ -29748,7 +29760,7 @@
       </c>
       <c r="F446" s="4" t="inlineStr">
         <is>
-          <t>Your next attack deals weapon DMG + 18. If you guarded an attack within the last 30 seconds, this deals weapon DMG + 30 instead.</t>
+          <t>Queue your next auto attack to deal weapon DMG + 18. If you guarded an attack within the last 30 seconds, it deals weapon DMG + 30 instead.</t>
         </is>
       </c>
       <c r="G446" s="3" t="inlineStr">
@@ -29763,7 +29775,7 @@
       </c>
       <c r="I446" s="3" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Queued</t>
         </is>
       </c>
       <c r="J446" s="3" t="inlineStr">
@@ -29778,7 +29790,7 @@
       </c>
       <c r="L446" s="12" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M446" s="13" t="inlineStr">
@@ -29790,7 +29802,11 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Add today's current date"")"),"2026-07-18")</f>
         <v/>
       </c>
-      <c r="O446" s="18" t="n"/>
+      <c r="O446" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Converted from a click-targeted activation to a self-queued weapon ability. It now applies to the next landed auto attack and no longer displays a target cursor. Regression retest required.</t>
+        </is>
+      </c>
     </row>
     <row r="447" ht="15" customHeight="1" s="16">
       <c r="A447" s="9" t="inlineStr">
@@ -29936,7 +29952,7 @@
       </c>
       <c r="O448" s="18" t="inlineStr">
         <is>
-          <t>See Discord // Developer follow-up (2026-07-19): Fixed the reported mismatch: the +15 DMG now pulses to hostile creatures within 5m and adds enmity equal to the guarded hit's incoming damage for additional targets. Secondary damage is non-recursive.</t>
+          <t>See Discord // Developer follow-up (2026-07-19): Fixed the reported mismatch: the +15 DMG now pulses to hostile creatures within 5m and adds enmity equal to the guarded hit's incoming damage for additional targets. Secondary damage is non-recursive. // Developer review (2026-07-19): The reported idle Guard events were valid incoming physical hits from the named enemies; Iron Guard Training is passive and Iron Elbows automatically pulses on Guard. Static guards reject invalid/self/zero/nonphysical events before rolling. Retest the separate engine log line showing 'Someone: 0' and capture target context if it persists.</t>
         </is>
       </c>
     </row>
@@ -30480,7 +30496,7 @@
       </c>
       <c r="F456" s="4" t="inlineStr">
         <is>
-          <t>Your next attack deals weapon DMG + 28. If you guarded an attack within the last 30 seconds, this deals weapon DMG + 45 instead and inflicts Dazed for 15 seconds.</t>
+          <t>Queue your next auto attack to deal weapon DMG + 28. If you guarded an attack within the last 30 seconds, it deals weapon DMG + 45 instead and inflicts Dazed for 15 seconds.</t>
         </is>
       </c>
       <c r="G456" s="3" t="inlineStr">
@@ -30495,7 +30511,7 @@
       </c>
       <c r="I456" s="3" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Queued</t>
         </is>
       </c>
       <c r="J456" s="3" t="inlineStr">
@@ -30510,7 +30526,7 @@
       </c>
       <c r="L456" s="12" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M456" s="13" t="inlineStr">
@@ -30522,7 +30538,11 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Add today's current date"")"),"2026-07-18")</f>
         <v/>
       </c>
-      <c r="O456" s="18" t="n"/>
+      <c r="O456" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Converted from a click-targeted activation to a self-queued weapon ability. It now applies to the next landed auto attack and no longer displays a target cursor. Regression retest required.</t>
+        </is>
+      </c>
     </row>
     <row r="457" ht="15" customHeight="1" s="16">
       <c r="A457" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Fix queued weapon impact animations
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -64095,12 +64095,16 @@
       </c>
       <c r="L969" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M969" s="13" t="n"/>
       <c r="N969" s="14" t="n"/>
-      <c r="O969" s="18" t="n"/>
+      <c r="O969" s="18" t="inlineStr">
+        <is>
+          <t>Retest queued Pathogen Strike on a normal attack that kills the target. Confirm the native attack animation plays once with no delayed extra swing after death. Also confirm nonlethal hits and Venom/Infection extension remain correct.</t>
+        </is>
+      </c>
     </row>
     <row r="970" ht="15" customHeight="1" s="16">
       <c r="A970" s="2" t="inlineStr">
@@ -64355,12 +64359,16 @@
       </c>
       <c r="L973" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M973" s="13" t="n"/>
       <c r="N973" s="14" t="n"/>
-      <c r="O973" s="18" t="n"/>
+      <c r="O973" s="18" t="inlineStr">
+        <is>
+          <t>Retest queued Pathogen Strike on a normal attack that kills the target. Confirm the native attack animation plays once with no delayed extra swing after death. Also confirm nonlethal hits and Venom/Infection extension remain correct.</t>
+        </is>
+      </c>
     </row>
     <row r="974" ht="15" customHeight="1" s="16">
       <c r="A974" s="2" t="inlineStr">
@@ -64745,12 +64753,16 @@
       </c>
       <c r="L979" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M979" s="13" t="n"/>
       <c r="N979" s="14" t="n"/>
-      <c r="O979" s="18" t="n"/>
+      <c r="O979" s="18" t="inlineStr">
+        <is>
+          <t>Retest queued Pathogen Strike on a normal attack that kills the target. Confirm the native attack animation plays once with no delayed extra swing after death. Also confirm nonlethal hits and Venom/Infection extension remain correct.</t>
+        </is>
+      </c>
     </row>
     <row r="980" ht="15" customHeight="1" s="16">
       <c r="A980" s="2" t="inlineStr">
@@ -65070,12 +65082,16 @@
       </c>
       <c r="L984" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M984" s="13" t="n"/>
       <c r="N984" s="14" t="n"/>
-      <c r="O984" s="18" t="n"/>
+      <c r="O984" s="18" t="inlineStr">
+        <is>
+          <t>Retest queued Pathogen Strike on a normal attack that kills the target. Confirm the native attack animation plays once with no delayed extra swing after death. Also confirm nonlethal hits and Venom/Infection extension remain correct.</t>
+        </is>
+      </c>
     </row>
     <row r="985" ht="15" customHeight="1" s="16">
       <c r="A985" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Correct guard retaliation DMG scaling
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -29984,7 +29984,7 @@
       </c>
       <c r="F449" s="17" t="inlineStr">
         <is>
-          <t>For 30 seconds, you gain +20 Guard and deal 8 DMG back to attackers whenever you guard a hit. Your current Guarded target automatically receives the same effect if they are within 5 meters.</t>
+          <t>For 30 seconds, you gain +20 Guard. Whenever you guard a hit, deal 8 physical DMG to that attacker using the standard combat damage formula. Your current Guarded target automatically receives the same effect if they are within 5 meters when activated.</t>
         </is>
       </c>
       <c r="G449" s="10" t="inlineStr">
@@ -30028,7 +30028,7 @@
       </c>
       <c r="O449" s="18" t="inlineStr">
         <is>
-          <t>Works but review damage calculation // Developer follow-up (2026-07-19): Corrected damage calculation: the stated 8 retaliation DMG is fixed, while Iron Elbows' separate +15 bonus uses the Katar combat formula. Regression retest required.</t>
+          <t>Works but review damage calculation // Developer correction (2026-07-20): DMG is a combat-rating input, not flat HP damage. Whirling Guard's 8 DMG and Iron Elbows' +15 DMG now resolve through the standard attack-versus-defense damage range per target, then use non-recursive triggered delivery. Regression retest required; retaliation values should vary with stats and target Defense.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make Retaliatory Flow cross-skill
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -30348,7 +30348,7 @@
       </c>
       <c r="F454" s="4" t="inlineStr">
         <is>
-          <t>After you guard a hit, your next Katar attack within 30 seconds deals +8 DMG.</t>
+          <t>After you guard a hit, your next attack within 30 seconds deals +8 DMG and generates +40 Enmity.</t>
         </is>
       </c>
       <c r="G454" s="3" t="inlineStr">
@@ -30392,7 +30392,7 @@
       </c>
       <c r="O454" s="18" t="inlineStr">
         <is>
-          <t>Developer follow-up (2026-07-19): Fixed its selector collision with Redirecting Counter and added shared 'Counter Ready' feedback. When both are owned, the next Katar attack correctly receives +18 DMG and +10% critical chance.</t>
+          <t>Developer follow-up (2026-07-20): Retaliatory Flow is now cross-skill. After Guard, the next attack within 30 seconds receives +8 DMG before attack-versus-defense resolution and generates +40 Enmity. When combined with Redirecting Counter, the shared next attack receives +18 DMG, +10% critical chance, and +40 Enmity; the window remains 30 seconds. Regression retest required with at least one non-Katar auto attack and one non-Katar hostile ability.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix High Guard costly ability interactions (#2102)
* Fix High Guard costly ability interactions

* Address High Guard review concerns

* Address deferred impact review findings
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -53495,7 +53495,7 @@
       </c>
       <c r="O809" s="18" t="inlineStr">
         <is>
-          <t>Did not grant evasion on trigger // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +3% Evasion for 30 seconds; damage remains +6.</t>
+          <t>Did not grant evasion on trigger // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +3% Evasion for 30 seconds; damage remains +6. // Developer correction (2026-07-19): The earlier fix was incomplete. Restoration Strike consumed the paid-cost context before High Guard Evasion ran, while shared minimum-cost stats made High Guard damage, Restoration Strike, and Crippling Defense thresholds add together. The cost is now bound to the exact ability, remains available to every independent rider, restores STM only once, and uses separate 8 STM thresholds. High Guard now applies globally per the Bible wording. Retest with Restoration Strike and Crippling Defense owned, using any hostile ability that spends at least 8 final STM.</t>
         </is>
       </c>
     </row>
@@ -53941,7 +53941,7 @@
       </c>
       <c r="O815" s="18" t="inlineStr">
         <is>
-          <t>No evasion increase, no way to tell DMG increased // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +5% Evasion for 30 seconds; damage remains +10.</t>
+          <t>No evasion increase, no way to tell DMG increased // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +5% Evasion for 30 seconds; damage remains +10. // Developer correction (2026-07-19): The earlier fix was incomplete. Restoration Strike consumed the paid-cost context before High Guard Evasion ran, while shared minimum-cost stats made High Guard damage, Restoration Strike, and Crippling Defense thresholds add together. The cost is now bound to the exact ability, remains available to every independent rider, restores STM only once, and uses separate 8 STM thresholds. High Guard now applies globally per the Bible wording. Retest with Restoration Strike and Crippling Defense owned, using any hostile ability that spends at least 8 final STM.</t>
         </is>
       </c>
     </row>
@@ -54003,7 +54003,7 @@
       </c>
       <c r="L816" s="12" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M816" s="13" t="inlineStr">
@@ -54015,7 +54015,11 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Fill with today's date"")"),"2026-07-18")</f>
         <v/>
       </c>
-      <c r="O816" s="18" t="n"/>
+      <c r="O816" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Corrected an interaction bug in the shared costly-ability context. Restoration Strike no longer raises High Guard's damage threshold, no longer consumes High Guard's Evasion trigger, restores 3 STM only once per ability, and now applies to any hostile ability spending at least 8 final STM as written. Retest together with High Guard and a multi-target ability.</t>
+        </is>
+      </c>
     </row>
     <row r="817" ht="15" customHeight="1" s="16">
       <c r="A817" s="9" t="inlineStr">
@@ -54537,7 +54541,7 @@
       </c>
       <c r="O823" s="18" t="inlineStr">
         <is>
-          <t>No evasion increase, no way to tell DMG increased // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +7% Evasion for 30 seconds; damage remains +14.</t>
+          <t>No evasion increase, no way to tell DMG increased // Developer follow-up (2026-07-19): Fixed the missing cost-gated Evasion trigger and isolated it from other Spear trigger channels. Hostile abilities that actually spend at least 8 STM now grant +7% Evasion for 30 seconds; damage remains +14. // Developer correction (2026-07-19): The earlier fix was incomplete. Restoration Strike consumed the paid-cost context before High Guard Evasion ran, while shared minimum-cost stats made High Guard damage, Restoration Strike, and Crippling Defense thresholds add together. The cost is now bound to the exact ability, remains available to every independent rider, restores STM only once, and uses separate 8 STM thresholds. High Guard now applies globally per the Bible wording. Retest with Restoration Strike and Crippling Defense owned, using any hostile ability that spends at least 8 final STM.</t>
         </is>
       </c>
     </row>
@@ -54613,7 +54617,7 @@
       </c>
       <c r="O824" s="18" t="inlineStr">
         <is>
-          <t>Ability locked // Developer follow-up (2026-07-19): No defect identified; this is the intended capstone quest gate. Retest with the quest completed or an approved admin test fixture.</t>
+          <t>Ability locked // Developer follow-up (2026-07-19): No defect identified; this is the intended capstone quest gate. Retest with the quest completed or an approved admin test fixture. // Developer follow-up (2026-07-19): Its 8 STM Exposed threshold is now independent rather than adding to High Guard/Restoration thresholds, and “high-STM abilities” is global per the Bible. Keep Blocked until capstone access is available; then retest alongside High Guard and Restoration Strike.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make Iron Elbows standalone and cross-skill
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -29908,7 +29908,7 @@
       </c>
       <c r="F448" s="4" t="inlineStr">
         <is>
-          <t>Iron Guard counterattacks and guard pulses deal +15 DMG to enemies within 5m and generate Enmity equal to the guarded hit's incoming damage.</t>
+          <t>Whenever you Guard a hostile hit, release a pulse that deals 15 physical DMG to the attacker and all other enemies within 5 meters, using the standard combat damage formula. Each affected enemy generates Enmity toward you equal to the guarded hit's incoming damage.</t>
         </is>
       </c>
       <c r="G448" s="3" t="inlineStr">
@@ -29952,7 +29952,7 @@
       </c>
       <c r="O448" s="18" t="inlineStr">
         <is>
-          <t>See Discord // Developer follow-up (2026-07-19): Fixed the reported mismatch: the +15 DMG now pulses to hostile creatures within 5m and adds enmity equal to the guarded hit's incoming damage for additional targets. Secondary damage is non-recursive. // Developer review (2026-07-19): The reported idle Guard events were valid incoming physical hits from the named enemies; Iron Guard Training is passive and Iron Elbows automatically pulses on Guard. Static guards reject invalid/self/zero/nonphysical events before rolling. Retest the separate engine log line showing 'Someone: 0' and capture target context if it persists.</t>
+          <t>See Discord // Developer follow-up (2026-07-19): Fixed the reported mismatch: the +15 DMG now pulses to hostile creatures within 5m and adds enmity equal to the guarded hit's incoming damage for additional targets. Secondary damage is non-recursive. // Developer review (2026-07-19): The reported idle Guard events were valid incoming physical hits from the named enemies; Iron Guard Training is passive and Iron Elbows automatically pulses on Guard. Static guards reject invalid/self/zero/nonphysical events before rolling. Retest the separate engine log line showing 'Someone: 0' and capture target context if it persists. // Developer follow-up (2026-07-20): Reworked Iron Elbows into a standalone cross-skill Guard trigger. Every successful hostile Guard now damages the triggering attacker regardless of range and other hostile creatures within 5 meters for 15 physical DMG through the standard combat formula. The triggering attacker receives normal Guard Enmity; each additional enemy hit receives Enmity equal to the guarded hit's incoming damage. The pulse requires no sibling perk, works with any weapon or unarmed, cannot double-hit the original attacker, and uses non-recursive damage delivery. Retest with Katar, a non-Katar weapon, unarmed, a ranged attacker beyond 5 meters, and multiple nearby enemies.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix stealth, guard counters, and outstanding combat feedback (#2106)
* Fix stealth and outstanding combat test feedback

* Fix guard counters and aimed area targeting

* Remove duplicate aimed area target handling

* Update resolved Guard Counter Haks assets

* Address final combat review feedback

* Fix queued weapon impact animations

* Clarify Whirling Guard fixed retaliation

* Correct guard retaliation DMG scaling

* Make Retaliatory Flow cross-skill

* Update Haks pointer after conflict resolution

* Address PR review findings

* Restore complete combat service after review fix

* Guard TLK synchronization conflicts

* Restore intended Combat Analyzer description

* Preserve telegraphed guarded-hit enmity

* Make Iron Elbows standalone and cross-skill

* Address CodeRabbit validation feedback

* Guard Combat Analyzer tier-neutral wording

* Label native party chat as Comms

* Separate area cursor and object targeting

* Simplify Guard damage descriptions
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -1280,7 +1280,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Increases Detection by 5, improving your chance to notice stealthed creatures.</t>
+          <t>Increases Detection by 10, improving your chance to notice stealthed creatures.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1310,12 +1310,16 @@
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M12" s="13" t="n"/>
       <c r="N12" s="14" t="n"/>
-      <c r="O12" s="18" t="n"/>
+      <c r="O12" s="18" t="inlineStr">
+        <is>
+          <t>Retest Detection = PER + WIL + equipment/status bonuses + 10 Alertness; Detect mode adds +5. Validate against all Stealth ranks at close and long visual range.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="16">
       <c r="A13" s="9" t="inlineStr">
@@ -1345,7 +1349,7 @@
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>Increases Detection by 10, improving your chance to notice stealthed creatures.</t>
+          <t>Increases Detection by 15, improving your chance to notice stealthed creatures.</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -1375,12 +1379,16 @@
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M13" s="13" t="n"/>
       <c r="N13" s="14" t="n"/>
-      <c r="O13" s="18" t="n"/>
+      <c r="O13" s="18" t="inlineStr">
+        <is>
+          <t>Retest Detection = PER + WIL + equipment/status bonuses + 15 Alertness; Detect mode adds +5. Validate against all Stealth ranks at close and long visual range.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="16">
       <c r="A14" s="2" t="inlineStr">
@@ -1410,7 +1418,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Increases Detection by 15, improving your chance to notice stealthed creatures.</t>
+          <t>Increases Detection by 20, improving your chance to notice stealthed creatures.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1440,12 +1448,16 @@
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="14" t="n"/>
-      <c r="O14" s="18" t="n"/>
+      <c r="O14" s="18" t="inlineStr">
+        <is>
+          <t>Retest Detection = PER + WIL + equipment/status bonuses + 20 Alertness; Detect mode adds +5. Validate that a fully committed spotter can counter a fully committed stealther.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="16">
       <c r="A15" s="9" t="inlineStr">
@@ -10737,12 +10749,16 @@
       </c>
       <c r="L157" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M157" s="13" t="n"/>
       <c r="N157" s="14" t="n"/>
-      <c r="O157" s="18" t="n"/>
+      <c r="O157" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Fixed the aimed-area activation contract. Adhesive Grenade I now explicitly requires the selected ground target supplied by its cursor; self-centered execution is rejected. Retest ground placement, the 4m blast, and the five-target cap.</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="15" customHeight="1" s="16">
       <c r="A158" s="2" t="inlineStr">
@@ -11128,12 +11144,16 @@
       </c>
       <c r="L163" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M163" s="13" t="n"/>
       <c r="N163" s="14" t="n"/>
-      <c r="O163" s="18" t="n"/>
+      <c r="O163" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Fixed the aimed-area activation contract. Adhesive Grenade II now explicitly requires the selected ground target supplied by its cursor; self-centered execution is rejected. Retest ground placement, the 4m blast, and the five-target cap.</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="15" customHeight="1" s="16">
       <c r="A164" s="2" t="inlineStr">
@@ -13284,7 +13304,11 @@
       <c r="N196" s="14" t="n">
         <v>46221</v>
       </c>
-      <c r="O196" s="18" t="n"/>
+      <c r="O196" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed intentional: Flamethrower I deals cone fire damage but does not apply Burn. Burn begins at Flamethrower II per the current Bible.</t>
+        </is>
+      </c>
     </row>
     <row r="197" ht="15" customHeight="1" s="16">
       <c r="A197" s="9" t="inlineStr">
@@ -13503,7 +13527,7 @@
       </c>
       <c r="O199" s="18" t="inlineStr">
         <is>
-          <t>Accuracy increase works, unclear if the crit boost does // Developer follow-up (2026-07-19): Verified +8% Assault Gadget Accuracy and +8% critical chance are consumed by every damaging Assault Gadget definition. Retest critical frequency with and without the perk.</t>
+          <t>Developer follow-up (2026-07-19): Fixed ability critical math so the 5% baseline and +8% Gadget Harness stack to 13% total. The Character Sheet now shows Assault Gadget Crit, and successful ability criticals print an identity-safe 'critically hits' combat message. With Tactical Uplink active, the displayed total should be 18%. Retest the readout and critical frequency over a large sample.</t>
         </is>
       </c>
     </row>
@@ -13649,7 +13673,7 @@
       </c>
       <c r="O201" s="18" t="inlineStr">
         <is>
-          <t>Burn effect seems to only last 1 round, burn duration not listed in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Burn (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Burn at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Flamethrower II on successful Burn applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -13795,7 +13819,7 @@
       </c>
       <c r="O203" s="18" t="inlineStr">
         <is>
-          <t>Bleed effect applies for 1 round, bleed duration not stated in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Bleed (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Bleed at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Rail Dart I on successful Bleed applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -13870,7 +13894,7 @@
       </c>
       <c r="O204" s="18" t="inlineStr">
         <is>
-          <t>Accuracy increase works, unclear if the crit boost does // Developer follow-up (2026-07-19): Verified the 30-second buff supplies +5% Devices ability Accuracy and +5% Devices ability critical chance, and Assault Gadgets consume both. Retest critical frequency with and without the buff.</t>
+          <t>Developer follow-up (2026-07-19): Fixed ability critical math so Tactical Uplink adds +5 points to the 5% baseline (10% without Gadget Harness; 18% with Harness). The Character Sheet Assault Gadget Crit row updates with the buff, and successful ability criticals print an identity-safe combat message. Retest the 30-second buff, readout, and critical frequency.</t>
         </is>
       </c>
     </row>
@@ -14304,7 +14328,7 @@
       </c>
       <c r="O210" s="18" t="inlineStr">
         <is>
-          <t>Burn effect seems to only last 1 round, burn duration not listed in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Burn (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Burn at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Flamethrower III on successful Burn applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -14379,7 +14403,7 @@
       </c>
       <c r="O211" s="18" t="inlineStr">
         <is>
-          <t>Bleed effect applies for 1 round, bleed duration not stated in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Bleed (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Bleed at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Rail Dart II on successful Bleed applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -14600,7 +14624,7 @@
       </c>
       <c r="O214" s="18" t="inlineStr">
         <is>
-          <t>Bleed effect applies for 1 round, bleed duration not stated in description // Developer follow-up (2026-07-19): Implementation and description now both specify a 12-second Bleed (two combat rounds). Retest duration on a successful status application.</t>
+          <t>Developer follow-up (2026-07-19): Fixed the shared NWN status-effect boundary race. The documented 12-second Bleed at 6-second frequency now has enough native lifetime to deliver both logical damage ticks. Retest Rail Dart III on successful Bleed applications; resistance can still prevent the status.</t>
         </is>
       </c>
     </row>
@@ -15500,7 +15524,7 @@
       </c>
       <c r="F228" s="4" t="inlineStr">
         <is>
-          <t>Enter stealth, increasing stealth effectiveness by 15% while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
+          <t>Enter stealth, increasing Stealth by 5 while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
         </is>
       </c>
       <c r="G228" s="3" t="inlineStr">
@@ -15530,12 +15554,16 @@
       </c>
       <c r="L228" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M228" s="13" t="n"/>
       <c r="N228" s="14" t="n"/>
-      <c r="O228" s="18" t="n"/>
+      <c r="O228" s="18" t="inlineStr">
+        <is>
+          <t>Retest base Stealth without the perk (no mode, status, or STM drain), perk toggle on/off, clean in-combat rejection, icon/drain cleanup, and Stealth = (AGI x 2) + equipment/status + 5.</t>
+        </is>
+      </c>
     </row>
     <row r="229" ht="15" customHeight="1" s="16">
       <c r="A229" s="9" t="inlineStr">
@@ -15760,7 +15788,7 @@
       </c>
       <c r="F232" s="4" t="inlineStr">
         <is>
-          <t>Enter stealth, increasing stealth effectiveness by 25% while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
+          <t>Enter stealth, increasing Stealth by 10 while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
         </is>
       </c>
       <c r="G232" s="3" t="inlineStr">
@@ -15790,12 +15818,16 @@
       </c>
       <c r="L232" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M232" s="13" t="n"/>
       <c r="N232" s="14" t="n"/>
-      <c r="O232" s="18" t="n"/>
+      <c r="O232" s="18" t="inlineStr">
+        <is>
+          <t>Retest toggle, clean in-combat rejection, icon/drain cleanup, hostile-action break, and Stealth = (AGI x 2) + equipment/status + 10.</t>
+        </is>
+      </c>
     </row>
     <row r="233" ht="15" customHeight="1" s="16">
       <c r="A233" s="9" t="inlineStr">
@@ -16020,7 +16052,7 @@
       </c>
       <c r="F236" s="4" t="inlineStr">
         <is>
-          <t>Enter stealth, increasing stealth effectiveness by 35% while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
+          <t>Enter stealth, increasing Stealth by 15 while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
         </is>
       </c>
       <c r="G236" s="3" t="inlineStr">
@@ -16050,12 +16082,16 @@
       </c>
       <c r="L236" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M236" s="13" t="n"/>
       <c r="N236" s="14" t="n"/>
-      <c r="O236" s="18" t="n"/>
+      <c r="O236" s="18" t="inlineStr">
+        <is>
+          <t>Retest toggle, clean in-combat rejection, icon/drain cleanup, hostile-action break, and Stealth = (AGI x 2) + equipment/status + 15 against groups of observers.</t>
+        </is>
+      </c>
     </row>
     <row r="237" ht="15" customHeight="1" s="16">
       <c r="A237" s="9" t="inlineStr">
@@ -16150,7 +16186,7 @@
       </c>
       <c r="F238" s="4" t="inlineStr">
         <is>
-          <t>Removes the movement-speed penalty from stealth and reduces its STM drain rate by 20%, from 2 STM every 6 seconds to 2 STM every 7.5 seconds.</t>
+          <t>While stealthed, increases Movement Speed by 30% and reduces STM drain by 20%, from 2 STM every 6 seconds to 2 STM every 7.5 seconds. Stealth still prevents running at full speed.</t>
         </is>
       </c>
       <c r="G238" s="3" t="inlineStr">
@@ -16180,12 +16216,16 @@
       </c>
       <c r="L238" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M238" s="13" t="n"/>
       <c r="N238" s="14" t="n"/>
-      <c r="O238" s="18" t="n"/>
+      <c r="O238" s="18" t="inlineStr">
+        <is>
+          <t>Retest immediate +30% Movement Speed on entering stealth without toggling walk, removal on stealth exit, retained running restriction, and 2 STM drain every 7.5 seconds.</t>
+        </is>
+      </c>
     </row>
     <row r="239" ht="15" customHeight="1" s="16">
       <c r="A239" s="9" t="inlineStr">
@@ -16345,7 +16385,7 @@
       </c>
       <c r="F241" s="17" t="inlineStr">
         <is>
-          <t>Enter stealth, increasing stealth effectiveness by 45% while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
+          <t>Enter stealth, increasing Stealth by 20 while active. Drains 2 STM every 6 seconds, breaks on hostile action, and can only be entered while out of combat.</t>
         </is>
       </c>
       <c r="G241" s="10" t="inlineStr">
@@ -16375,12 +16415,16 @@
       </c>
       <c r="L241" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M241" s="13" t="n"/>
       <c r="N241" s="14" t="n"/>
-      <c r="O241" s="18" t="n"/>
+      <c r="O241" s="18" t="inlineStr">
+        <is>
+          <t>Retest toggle, clean in-combat rejection, icon/drain cleanup, hostile-action break, and Stealth = (AGI x 2) + equipment/status + 20. Validate committed stealth versus baseline monsters and committed spotters.</t>
+        </is>
+      </c>
     </row>
     <row r="242" ht="15" customHeight="1" s="16">
       <c r="A242" s="2" t="inlineStr">
@@ -16635,12 +16679,16 @@
       </c>
       <c r="L245" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M245" s="13" t="n"/>
       <c r="N245" s="14" t="n"/>
-      <c r="O245" s="18" t="n"/>
+      <c r="O245" s="18" t="inlineStr">
+        <is>
+          <t>Retest in-combat stealth entry through the explicit Ghost Protocol window, 30-second exit, status/icon cleanup, and the revised Stealth/Detection ratings.</t>
+        </is>
+      </c>
     </row>
     <row r="246" ht="15" customHeight="1" s="16">
       <c r="A246" s="2" t="inlineStr">
@@ -29416,7 +29464,7 @@
       </c>
       <c r="F442" s="4" t="inlineStr">
         <is>
-          <t>Your next attack deals weapon DMG + 8. If you guarded an attack within the last 30 seconds, this deals weapon DMG + 16 instead.</t>
+          <t>Queue your next auto attack to deal weapon DMG + 8. If you guarded an attack within the last 30 seconds, it deals weapon DMG + 16 instead.</t>
         </is>
       </c>
       <c r="G442" s="3" t="inlineStr">
@@ -29431,7 +29479,7 @@
       </c>
       <c r="I442" s="3" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Queued</t>
         </is>
       </c>
       <c r="J442" s="3" t="inlineStr">
@@ -29446,7 +29494,7 @@
       </c>
       <c r="L442" s="12" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M442" s="13" t="inlineStr">
@@ -29458,7 +29506,11 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Add today's current date"")"),"2026-07-18")</f>
         <v/>
       </c>
-      <c r="O442" s="18" t="n"/>
+      <c r="O442" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Converted from a click-targeted activation to a self-queued weapon ability. It now applies to the next landed auto attack and no longer displays a target cursor. Regression retest required.</t>
+        </is>
+      </c>
     </row>
     <row r="443" ht="15" customHeight="1" s="16">
       <c r="A443" s="9" t="inlineStr">
@@ -29560,7 +29612,7 @@
       </c>
       <c r="F444" s="4" t="inlineStr">
         <is>
-          <t>When you guard an attack, your next Katar attack within 30 seconds gains +10% critical chance and deals +10 DMG.</t>
+          <t>When you guard an attack, your next attack within 30 seconds gains +10% critical chance and deals +10 DMG.</t>
         </is>
       </c>
       <c r="G444" s="3" t="inlineStr">
@@ -29604,7 +29656,7 @@
       </c>
       <c r="O444" s="18" t="inlineStr">
         <is>
-          <t>No feedback to tell if triggering // Developer follow-up (2026-07-19): Added explicit 'Counter Ready' feedback. Also fixed its selector collision with Retaliatory Flow so both perks combine as +18 DMG and +10% critical chance instead of producing an invalid skill ID.</t>
+          <t>No feedback to tell if triggering // Developer follow-up (2026-07-19): Added explicit 'Counter Ready' feedback. Also fixed its selector collision with Retaliatory Flow so both perks combine as +18 DMG and +10% critical chance instead of producing an invalid skill ID. // Developer follow-up (2026-07-19): Reworked the trigger to be cross-skill. Guard now arms the next hostile combat ability from any skill with +10 DMG and +10% critical chance for 30 seconds; friendly/self abilities do not consume it. Regression retest required.</t>
         </is>
       </c>
     </row>
@@ -29708,7 +29760,7 @@
       </c>
       <c r="F446" s="4" t="inlineStr">
         <is>
-          <t>Your next attack deals weapon DMG + 18. If you guarded an attack within the last 30 seconds, this deals weapon DMG + 30 instead.</t>
+          <t>Queue your next auto attack to deal weapon DMG + 18. If you guarded an attack within the last 30 seconds, it deals weapon DMG + 30 instead.</t>
         </is>
       </c>
       <c r="G446" s="3" t="inlineStr">
@@ -29723,7 +29775,7 @@
       </c>
       <c r="I446" s="3" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Queued</t>
         </is>
       </c>
       <c r="J446" s="3" t="inlineStr">
@@ -29738,7 +29790,7 @@
       </c>
       <c r="L446" s="12" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M446" s="13" t="inlineStr">
@@ -29750,7 +29802,11 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Add today's current date"")"),"2026-07-18")</f>
         <v/>
       </c>
-      <c r="O446" s="18" t="n"/>
+      <c r="O446" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Converted from a click-targeted activation to a self-queued weapon ability. It now applies to the next landed auto attack and no longer displays a target cursor. Regression retest required.</t>
+        </is>
+      </c>
     </row>
     <row r="447" ht="15" customHeight="1" s="16">
       <c r="A447" s="9" t="inlineStr">
@@ -29852,7 +29908,7 @@
       </c>
       <c r="F448" s="4" t="inlineStr">
         <is>
-          <t>Iron Guard counterattacks and guard pulses deal +15 DMG to enemies within 5m and generate Enmity equal to the guarded hit's incoming damage.</t>
+          <t>Whenever you Guard a hostile hit, release a pulse that deals 15 physical DMG to the attacker and all other enemies within 5 meters, using the standard combat damage formula. Each affected enemy generates Enmity toward you equal to the guarded hit's incoming damage.</t>
         </is>
       </c>
       <c r="G448" s="3" t="inlineStr">
@@ -29896,7 +29952,7 @@
       </c>
       <c r="O448" s="18" t="inlineStr">
         <is>
-          <t>See Discord // Developer follow-up (2026-07-19): Fixed the reported mismatch: the +15 DMG now pulses to hostile creatures within 5m and adds enmity equal to the guarded hit's incoming damage for additional targets. Secondary damage is non-recursive.</t>
+          <t>See Discord // Developer follow-up (2026-07-19): Fixed the reported mismatch: the +15 DMG now pulses to hostile creatures within 5m and adds enmity equal to the guarded hit's incoming damage for additional targets. Secondary damage is non-recursive. // Developer review (2026-07-19): The reported idle Guard events were valid incoming physical hits from the named enemies; Iron Guard Training is passive and Iron Elbows automatically pulses on Guard. Static guards reject invalid/self/zero/nonphysical events before rolling. Retest the separate engine log line showing 'Someone: 0' and capture target context if it persists. // Developer follow-up (2026-07-20): Reworked Iron Elbows into a standalone cross-skill Guard trigger. Every successful hostile Guard now damages the triggering attacker regardless of range and other hostile creatures within 5 meters for 15 physical DMG through the standard combat formula. The triggering attacker receives normal Guard Enmity; each additional enemy hit receives Enmity equal to the guarded hit's incoming damage. The pulse requires no sibling perk, works with any weapon or unarmed, cannot double-hit the original attacker, and uses non-recursive damage delivery. Retest with Katar, a non-Katar weapon, unarmed, a ranged attacker beyond 5 meters, and multiple nearby enemies.</t>
         </is>
       </c>
     </row>
@@ -29928,7 +29984,7 @@
       </c>
       <c r="F449" s="17" t="inlineStr">
         <is>
-          <t>For 30 seconds, you gain +20 Guard and deal 8 DMG back to attackers whenever you guard a hit. Your current Guarded target automatically receives the same effect if they are within 5 meters.</t>
+          <t>For 30 seconds, you gain +20 Guard. Whenever you guard a hit, deal 8 physical DMG to that attacker using the standard combat damage formula. Your current Guarded target automatically receives the same effect if they are within 5 meters when activated.</t>
         </is>
       </c>
       <c r="G449" s="10" t="inlineStr">
@@ -29972,7 +30028,7 @@
       </c>
       <c r="O449" s="18" t="inlineStr">
         <is>
-          <t>Works but review damage calculation // Developer follow-up (2026-07-19): Corrected damage calculation: the stated 8 retaliation DMG is fixed, while Iron Elbows' separate +15 bonus uses the Katar combat formula. Regression retest required.</t>
+          <t>Works but review damage calculation // Developer correction (2026-07-20): DMG is a combat-rating input, not flat HP damage. Whirling Guard's 8 DMG and Iron Elbows' +15 DMG now resolve through the standard attack-versus-defense damage range per target, then use non-recursive triggered delivery. Regression retest required; retaliation values should vary with stats and target Defense.</t>
         </is>
       </c>
     </row>
@@ -30292,7 +30348,7 @@
       </c>
       <c r="F454" s="4" t="inlineStr">
         <is>
-          <t>After you guard a hit, your next Katar attack within 30 seconds deals +8 DMG.</t>
+          <t>After you guard a hit, your next attack within 30 seconds deals +8 DMG and generates +40 Enmity.</t>
         </is>
       </c>
       <c r="G454" s="3" t="inlineStr">
@@ -30336,7 +30392,7 @@
       </c>
       <c r="O454" s="18" t="inlineStr">
         <is>
-          <t>Developer follow-up (2026-07-19): Fixed its selector collision with Redirecting Counter and added shared 'Counter Ready' feedback. When both are owned, the next Katar attack correctly receives +18 DMG and +10% critical chance.</t>
+          <t>Developer follow-up (2026-07-20): Retaliatory Flow is now cross-skill. After Guard, the next attack within 30 seconds receives +8 DMG before attack-versus-defense resolution and generates +40 Enmity. When combined with Redirecting Counter, the shared next attack receives +18 DMG, +10% critical chance, and +40 Enmity; the window remains 30 seconds. Regression retest required with at least one non-Katar auto attack and one non-Katar hostile ability.</t>
         </is>
       </c>
     </row>
@@ -30440,7 +30496,7 @@
       </c>
       <c r="F456" s="4" t="inlineStr">
         <is>
-          <t>Your next attack deals weapon DMG + 28. If you guarded an attack within the last 30 seconds, this deals weapon DMG + 45 instead and inflicts Dazed for 15 seconds.</t>
+          <t>Queue your next auto attack to deal weapon DMG + 28. If you guarded an attack within the last 30 seconds, it deals weapon DMG + 45 instead and inflicts Dazed for 15 seconds.</t>
         </is>
       </c>
       <c r="G456" s="3" t="inlineStr">
@@ -30455,7 +30511,7 @@
       </c>
       <c r="I456" s="3" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Queued</t>
         </is>
       </c>
       <c r="J456" s="3" t="inlineStr">
@@ -30470,7 +30526,7 @@
       </c>
       <c r="L456" s="12" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M456" s="13" t="inlineStr">
@@ -30482,7 +30538,11 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("AI(""Add today's current date"")"),"2026-07-18")</f>
         <v/>
       </c>
-      <c r="O456" s="18" t="n"/>
+      <c r="O456" s="18" t="inlineStr">
+        <is>
+          <t>Developer follow-up (2026-07-19): Converted from a click-targeted activation to a self-queued weapon ability. It now applies to the next landed auto attack and no longer displays a target cursor. Regression retest required.</t>
+        </is>
+      </c>
     </row>
     <row r="457" ht="15" customHeight="1" s="16">
       <c r="A457" s="9" t="inlineStr">
@@ -64039,12 +64099,16 @@
       </c>
       <c r="L969" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M969" s="13" t="n"/>
       <c r="N969" s="14" t="n"/>
-      <c r="O969" s="18" t="n"/>
+      <c r="O969" s="18" t="inlineStr">
+        <is>
+          <t>Retest queued Pathogen Strike on a normal attack that kills the target. Confirm the native attack animation plays once with no delayed extra swing after death. Also confirm nonlethal hits and Venom/Infection extension remain correct.</t>
+        </is>
+      </c>
     </row>
     <row r="970" ht="15" customHeight="1" s="16">
       <c r="A970" s="2" t="inlineStr">
@@ -64299,12 +64363,16 @@
       </c>
       <c r="L973" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M973" s="13" t="n"/>
       <c r="N973" s="14" t="n"/>
-      <c r="O973" s="18" t="n"/>
+      <c r="O973" s="18" t="inlineStr">
+        <is>
+          <t>Retest queued Pathogen Strike on a normal attack that kills the target. Confirm the native attack animation plays once with no delayed extra swing after death. Also confirm nonlethal hits and Venom/Infection extension remain correct.</t>
+        </is>
+      </c>
     </row>
     <row r="974" ht="15" customHeight="1" s="16">
       <c r="A974" s="2" t="inlineStr">
@@ -64689,12 +64757,16 @@
       </c>
       <c r="L979" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M979" s="13" t="n"/>
       <c r="N979" s="14" t="n"/>
-      <c r="O979" s="18" t="n"/>
+      <c r="O979" s="18" t="inlineStr">
+        <is>
+          <t>Retest queued Pathogen Strike on a normal attack that kills the target. Confirm the native attack animation plays once with no delayed extra swing after death. Also confirm nonlethal hits and Venom/Infection extension remain correct.</t>
+        </is>
+      </c>
     </row>
     <row r="980" ht="15" customHeight="1" s="16">
       <c r="A980" s="2" t="inlineStr">
@@ -65014,12 +65086,16 @@
       </c>
       <c r="L984" s="12" t="inlineStr">
         <is>
-          <t>Not Tested</t>
+          <t>Retest</t>
         </is>
       </c>
       <c r="M984" s="13" t="n"/>
       <c r="N984" s="14" t="n"/>
-      <c r="O984" s="18" t="n"/>
+      <c r="O984" s="18" t="inlineStr">
+        <is>
+          <t>Retest queued Pathogen Strike on a normal attack that kills the target. Confirm the native attack animation plays once with no delayed extra swing after death. Also confirm nonlethal hits and Venom/Infection extension remain correct.</t>
+        </is>
+      </c>
     </row>
     <row r="985" ht="15" customHeight="1" s="16">
       <c r="A985" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Address Codex combat audit review
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -33072,8 +33072,7 @@
       </c>
       <c r="F495" s="17" t="inlineStr">
         <is>
-          <t>Enemies within Leadership range (5m base) suffer Flash for 30 seconds, reducing physical and Force ability hit chance by 10%.
-SOC scaling can raise the penalty to 12%. This command applies reliably to valid enemies within Leadership range (5m base).</t>
+          <t>Enemies within Leadership range (5m base) suffer Flash for 30 seconds, reducing Ability Accuracy by 10%. SOC scaling can raise the penalty to 12%. This command applies reliably to valid enemies within Leadership range (5m base).</t>
         </is>
       </c>
       <c r="G495" s="10" t="inlineStr">
@@ -33465,7 +33464,7 @@
       </c>
       <c r="F501" s="17" t="inlineStr">
         <is>
-          <t>Enemies within Leadership range (5m base) suffer Flash, reducing physical and Force ability hit chance by 15%, and Weakened, reducing Attack by 12%, for 30 seconds. SOC scaling can raise these penalties to 18% and 15%. This command applies reliably to valid enemies within Leadership range (5m base).</t>
+          <t>Enemies within Leadership range (5m base) suffer Flash, reducing Ability Accuracy by 15%, and Weakened, reducing Attack by 12%, for 30 seconds. SOC scaling can raise these penalties to 18% and 15%. This command applies reliably to valid enemies within Leadership range (5m base).</t>
         </is>
       </c>
       <c r="G501" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Fix combat testing tracker failures (#2200)
* Fix combat testing tracker failures

* Address Codex combat audit review
</commit_message>
<xml_diff>
--- a/design/testing/SWLOR CU Testing Tracker.xlsx
+++ b/design/testing/SWLOR CU Testing Tracker.xlsx
@@ -33072,8 +33072,7 @@
       </c>
       <c r="F495" s="17" t="inlineStr">
         <is>
-          <t>Enemies within Leadership range (5m base) suffer Flash for 30 seconds, reducing physical and Force ability hit chance by 10%.
-SOC scaling can raise the penalty to 12%. This command applies reliably to valid enemies within Leadership range (5m base).</t>
+          <t>Enemies within Leadership range (5m base) suffer Flash for 30 seconds, reducing Ability Accuracy by 10%. SOC scaling can raise the penalty to 12%. This command applies reliably to valid enemies within Leadership range (5m base).</t>
         </is>
       </c>
       <c r="G495" s="10" t="inlineStr">
@@ -33465,7 +33464,7 @@
       </c>
       <c r="F501" s="17" t="inlineStr">
         <is>
-          <t>Enemies within Leadership range (5m base) suffer Flash, reducing physical and Force ability hit chance by 15%, and Weakened, reducing Attack by 12%, for 30 seconds. SOC scaling can raise these penalties to 18% and 15%. This command applies reliably to valid enemies within Leadership range (5m base).</t>
+          <t>Enemies within Leadership range (5m base) suffer Flash, reducing Ability Accuracy by 15%, and Weakened, reducing Attack by 12%, for 30 seconds. SOC scaling can raise these penalties to 18% and 15%. This command applies reliably to valid enemies within Leadership range (5m base).</t>
         </is>
       </c>
       <c r="G501" s="10" t="inlineStr">

</xml_diff>